<commit_message>
fix: resolve bulk upload validation issues and style excel templates
</commit_message>
<xml_diff>
--- a/frontend/public/templates/sample_image_mcq_upload.xlsx
+++ b/frontend/public/templates/sample_image_mcq_upload.xlsx
@@ -26,9 +26,10 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="12"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
     </font>
   </fonts>
   <fills count="3">
@@ -54,28 +55,21 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="00000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="00000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="00000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00000000"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -444,16 +438,16 @@
   <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19.2" customWidth="1" min="1" max="1"/>
-    <col width="22.8" customWidth="1" min="2" max="2"/>
-    <col width="10.8" customWidth="1" min="3" max="3"/>
-    <col width="20.4" customWidth="1" min="4" max="4"/>
-    <col width="21.6" customWidth="1" min="5" max="5"/>
-    <col width="20.4" customWidth="1" min="6" max="6"/>
-    <col width="21.6" customWidth="1" min="7" max="7"/>
-    <col width="20.4" customWidth="1" min="8" max="8"/>
-    <col width="21.6" customWidth="1" min="9" max="9"/>
-    <col width="21.6" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="47" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -509,51 +503,45 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>APTITUDE</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>FRESHER</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Identify logo</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>logo.png</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>g.png</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Apple</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>a.png</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>1</v>
+      <c r="C2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Identify the object in the provided image.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>beautiful-cat.png</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>A fluffy cat</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>A golden retriever</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: optimize bulk upload service with Pydantic schemas and add sample templates for various question types.
</commit_message>
<xml_diff>
--- a/frontend/public/templates/sample_image_mcq_upload.xlsx
+++ b/frontend/public/templates/sample_image_mcq_upload.xlsx
@@ -26,10 +26,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="13"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="3">
@@ -41,8 +40,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F96331"/>
-        <bgColor rgb="00F96331"/>
+        <fgColor rgb="00f96331"/>
+        <bgColor rgb="00f96331"/>
       </patternFill>
     </fill>
   </fills>
@@ -64,12 +63,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -438,9 +436,9 @@
   <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="47" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
@@ -503,45 +501,41 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>APTITUDE</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>FRESHER</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" t="n">
         <v>5</v>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Identify the object in the provided image.</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>beautiful-cat.png</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>A fluffy cat</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>A golden retriever</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="J2" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add validator to coerce empty question inputs to None and update bulk upload template files
</commit_message>
<xml_diff>
--- a/frontend/public/templates/sample_image_mcq_upload.xlsx
+++ b/frontend/public/templates/sample_image_mcq_upload.xlsx
@@ -444,20 +444,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="41" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="41" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -493,25 +497,45 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Option 1 Image</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Option 2</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Option 2 Image</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Option 3</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Option 3 Image</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Option 4</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Option 4 Image</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Correct Option</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Explanation</t>
         </is>
@@ -536,35 +560,51 @@
           <t>Referencing visual dataset 1, identify the peak month.</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>data_chart_1.png</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>January</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>March</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>data_chart_2.png</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>June</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>data_chart_3.png</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>December</t>
         </is>
       </c>
-      <c r="J2" s="2" t="n">
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>data_chart_4.png</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>The chart clearly shows a peak in June.</t>
         </is>
@@ -589,35 +629,51 @@
           <t>Referencing visual dataset 2, identify the peak month.</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>data_chart_1.png</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>March</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>data_chart_2.png</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>January</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>March</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>June</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>data_chart_3.png</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>December</t>
         </is>
       </c>
-      <c r="J3" s="2" t="n">
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>data_chart_4.png</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>The chart clearly shows a peak in June.</t>
         </is>
@@ -642,35 +698,51 @@
           <t>Referencing visual dataset 3, identify the peak month.</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>data_chart_1.png</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>March</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>data_chart_2.png</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>June</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>data_chart_3.png</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>January</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>March</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>June</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>December</t>
         </is>
       </c>
-      <c r="J4" s="2" t="n">
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>data_chart_4.png</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>The chart clearly shows a peak in June.</t>
         </is>
@@ -695,35 +767,51 @@
           <t>Referencing visual dataset 4, identify the peak month.</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>data_chart_1.png</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>March</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>data_chart_2.png</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>June</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>data_chart_3.png</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>December</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>data_chart_4.png</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>January</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>March</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>June</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>December</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="n">
+      <c r="N5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>The chart clearly shows a peak in June.</t>
         </is>
@@ -748,11 +836,7 @@
           <t>Referencing visual dataset 5, identify the peak month.</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>data_chart_5.png</t>
-        </is>
-      </c>
+      <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>January</t>
@@ -760,23 +844,43 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
+          <t>data_chart_1.png</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
           <t>March</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>data_chart_2.png</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>June</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>data_chart_3.png</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>December</t>
         </is>
       </c>
-      <c r="J6" s="2" t="n">
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>data_chart_4.png</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>The chart clearly shows a peak in June.</t>
         </is>

</xml_diff>